<commit_message>
n8n board refresh 2026-10-16T17:41:44Z
</commit_message>
<xml_diff>
--- a/app/reports/IMSR_research.xlsx
+++ b/app/reports/IMSR_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-15 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-16 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>3.075</v>
+        <v>3.085</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.05085000038146972</v>
+        <v>0.05105999946594238</v>
       </c>
     </row>
     <row r="6">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>105935255.9349593</v>
+        <v>105935258.3468395</v>
       </c>
     </row>
     <row r="36">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>3.075</v>
+        <v>3.085</v>
       </c>
     </row>
     <row r="38">
@@ -1493,11 +1493,11 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>325750912</v>
+        <v>326810272</v>
       </c>
       <c r="D5" s="31" t="n"/>
       <c r="E5" s="31" t="n">
-        <v>-1.11</v>
+        <v>-1.89</v>
       </c>
       <c r="F5" s="31" t="n"/>
     </row>
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>539930624</v>
+        <v>531470144</v>
       </c>
       <c r="D6" s="33" t="n"/>
       <c r="E6" s="33" t="n">
-        <v>12.268</v>
+        <v>12.513</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>1.236</v>
+        <v>1.26</v>
       </c>
     </row>
     <row r="7">
@@ -1535,14 +1535,14 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>696960192</v>
+        <v>685078208</v>
       </c>
       <c r="D7" s="33" t="n"/>
       <c r="E7" s="33" t="n">
-        <v>12.812</v>
+        <v>12.838</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>1.61</v>
+        <v>1.613</v>
       </c>
     </row>
     <row r="8">
@@ -1557,16 +1557,16 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>1582742912</v>
+        <v>1525405056</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>15.816216</v>
+        <v>14.842106</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>12.547</v>
+        <v>12.321</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>8.321</v>
+        <v>8.170999999999999</v>
       </c>
     </row>
     <row r="9">
@@ -1581,16 +1581,16 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>1984434048</v>
+        <v>2045359616</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>15.199999</v>
+        <v>14.920634</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>6.474</v>
+        <v>6.454</v>
       </c>
       <c r="F9" s="33" t="n">
-        <v>2.598</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="10">
@@ -1605,16 +1605,16 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>1928130688</v>
+        <v>1967644416</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>32.05814</v>
+        <v>31.61236</v>
       </c>
       <c r="E10" s="33" t="n">
-        <v>10.26</v>
+        <v>10.072</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>1.798</v>
+        <v>1.765</v>
       </c>
     </row>
     <row r="11">
@@ -1629,16 +1629,16 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>2048468480</v>
+        <v>2079311232</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>18.75294</v>
+        <v>19.035294</v>
       </c>
       <c r="E11" s="33" t="n">
-        <v>8.801</v>
+        <v>8.864000000000001</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>6.621</v>
+        <v>6.668</v>
       </c>
     </row>
     <row r="12">
@@ -1653,14 +1653,14 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>513924000</v>
+        <v>519623680</v>
       </c>
       <c r="D12" s="33" t="n"/>
       <c r="E12" s="33" t="n">
-        <v>-189.251</v>
+        <v>-189.083</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>1.392</v>
+        <v>1.391</v>
       </c>
     </row>
     <row r="13">
@@ -1676,13 +1676,13 @@
       </c>
       <c r="C13" s="32" t="n"/>
       <c r="D13" s="33" t="n">
-        <v>14.206409</v>
+        <v>14.190063</v>
       </c>
       <c r="E13" s="33" t="n">
-        <v>9.685</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>7.433</v>
+        <v>7.46</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-10-17T17:41:03Z
</commit_message>
<xml_diff>
--- a/app/reports/IMSR_research.xlsx
+++ b/app/reports/IMSR_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-16 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-17 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>3.085</v>
+        <v>3.05</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.05105999946594238</v>
+        <v>0.05098000049591064</v>
       </c>
     </row>
     <row r="6">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>105935258.3468395</v>
+        <v>105935255.0819672</v>
       </c>
     </row>
     <row r="36">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>3.085</v>
+        <v>3.05</v>
       </c>
     </row>
     <row r="38">
@@ -1493,11 +1493,11 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>326810272</v>
+        <v>323102528</v>
       </c>
       <c r="D5" s="31" t="n"/>
       <c r="E5" s="31" t="n">
-        <v>-1.89</v>
+        <v>-1.42</v>
       </c>
       <c r="F5" s="31" t="n"/>
     </row>
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>531470144</v>
+        <v>527624512</v>
       </c>
       <c r="D6" s="33" t="n"/>
       <c r="E6" s="33" t="n">
-        <v>12.513</v>
+        <v>12.333</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>1.26</v>
+        <v>1.242</v>
       </c>
     </row>
     <row r="7">
@@ -1535,14 +1535,14 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>685078208</v>
+        <v>666067136</v>
       </c>
       <c r="D7" s="33" t="n"/>
       <c r="E7" s="33" t="n">
-        <v>12.838</v>
+        <v>12.755</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>1.613</v>
+        <v>1.602</v>
       </c>
     </row>
     <row r="8">
@@ -1557,16 +1557,16 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>1525405056</v>
+        <v>1527027712</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>14.842106</v>
+        <v>14.857895</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>12.321</v>
+        <v>12.228</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>8.170999999999999</v>
+        <v>8.109999999999999</v>
       </c>
     </row>
     <row r="9">
@@ -1581,16 +1581,16 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>2045359616</v>
+        <v>2046447616</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>14.920634</v>
+        <v>14.928571</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>6.454</v>
+        <v>6.518</v>
       </c>
       <c r="F9" s="33" t="n">
-        <v>2.59</v>
+        <v>2.616</v>
       </c>
     </row>
     <row r="10">
@@ -1605,16 +1605,16 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>1967644416</v>
+        <v>1960301184</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>31.61236</v>
+        <v>31.494383</v>
       </c>
       <c r="E10" s="33" t="n">
-        <v>10.072</v>
+        <v>10.328</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>1.765</v>
+        <v>1.809</v>
       </c>
     </row>
     <row r="11">
@@ -1629,16 +1629,16 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>2079311232</v>
+        <v>2092162432</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>19.035294</v>
+        <v>19.15294</v>
       </c>
       <c r="E11" s="33" t="n">
-        <v>8.864000000000001</v>
+        <v>8.996</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>6.668</v>
+        <v>6.768</v>
       </c>
     </row>
     <row r="12">
@@ -1653,14 +1653,14 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>519623680</v>
+        <v>498640000</v>
       </c>
       <c r="D12" s="33" t="n"/>
       <c r="E12" s="33" t="n">
-        <v>-189.083</v>
+        <v>-180.518</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>1.391</v>
+        <v>1.328</v>
       </c>
     </row>
     <row r="13">
@@ -1676,13 +1676,13 @@
       </c>
       <c r="C13" s="32" t="n"/>
       <c r="D13" s="33" t="n">
-        <v>14.190063</v>
+        <v>14.345663</v>
       </c>
       <c r="E13" s="33" t="n">
-        <v>9.720000000000001</v>
+        <v>9.792999999999999</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>7.46</v>
+        <v>7.516</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-10-19T17:41:33Z
</commit_message>
<xml_diff>
--- a/app/reports/IMSR_research.xlsx
+++ b/app/reports/IMSR_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-18 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-19 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>3.05</v>
+        <v>2.905</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.05098000049591064</v>
+        <v>0.0514799976348877</v>
       </c>
     </row>
     <row r="6">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>105935255.0819672</v>
+        <v>105935256.454389</v>
       </c>
     </row>
     <row r="36">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>3.05</v>
+        <v>2.905</v>
       </c>
     </row>
     <row r="38">
@@ -1493,7 +1493,7 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>323102528</v>
+        <v>307741920</v>
       </c>
       <c r="D5" s="31" t="n"/>
       <c r="E5" s="31" t="n">
@@ -1513,7 +1513,7 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>527624512</v>
+        <v>494551808</v>
       </c>
       <c r="D6" s="33" t="n"/>
       <c r="E6" s="33" t="n">
@@ -1535,7 +1535,7 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>666067136</v>
+        <v>635174080</v>
       </c>
       <c r="D7" s="33" t="n"/>
       <c r="E7" s="33" t="n">
@@ -1557,10 +1557,10 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>1527027712</v>
+        <v>1483753856</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>14.857895</v>
+        <v>14.436843</v>
       </c>
       <c r="E8" s="33" t="n">
         <v>12.228</v>
@@ -1581,10 +1581,10 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>2046447616</v>
+        <v>2051887488</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>14.928571</v>
+        <v>14.968254</v>
       </c>
       <c r="E9" s="33" t="n">
         <v>6.518</v>
@@ -1605,10 +1605,10 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>1960301184</v>
+        <v>1956412672</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>31.494383</v>
+        <v>31.43191</v>
       </c>
       <c r="E10" s="33" t="n">
         <v>10.328</v>
@@ -1629,10 +1629,10 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>2092162432</v>
+        <v>2095375104</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>19.15294</v>
+        <v>19.182352</v>
       </c>
       <c r="E11" s="33" t="n">
         <v>8.996</v>
@@ -1653,7 +1653,7 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>498640000</v>
+        <v>495455872</v>
       </c>
       <c r="D12" s="33" t="n"/>
       <c r="E12" s="33" t="n">
@@ -1676,7 +1676,7 @@
       </c>
       <c r="C13" s="32" t="n"/>
       <c r="D13" s="33" t="n">
-        <v>14.345663</v>
+        <v>14.47704</v>
       </c>
       <c r="E13" s="33" t="n">
         <v>9.792999999999999</v>

</xml_diff>